<commit_message>
I accidentally counted the same samples twice....
</commit_message>
<xml_diff>
--- a/data/raw/Cell_Counts/Dazl_100nMRA/241009_Dazl_100nMRA.xlsx
+++ b/data/raw/Cell_Counts/Dazl_100nMRA/241009_Dazl_100nMRA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://umhealth-my.sharepoint.com/personal/kbonefas_med_umich_edu/Documents/Documents/KDM5C_Germ_Mechanism/data/raw/Cell_Counts/Dazl_100nMRA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="498" documentId="11_F25DC773A252ABDACC1048D6E9986E465BDE58ED" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A4DF3129-7585-4282-8E80-6483899DBAB4}"/>
+  <xr:revisionPtr revIDLastSave="542" documentId="11_F25DC773A252ABDACC1048D6E9986E465BDE58ED" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4D9271E9-4378-4154-BE31-D00EFEE944CE}"/>
   <bookViews>
-    <workbookView xWindow="4800" yWindow="340" windowWidth="14400" windowHeight="7270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="483" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="418" uniqueCount="22">
   <si>
     <t>Image</t>
   </si>
@@ -70,6 +70,27 @@
   </si>
   <si>
     <t>WT</t>
+  </si>
+  <si>
+    <t>H3</t>
+  </si>
+  <si>
+    <t>I3</t>
+  </si>
+  <si>
+    <t>J3</t>
+  </si>
+  <si>
+    <t>G1</t>
+  </si>
+  <si>
+    <t>H1</t>
+  </si>
+  <si>
+    <t>I1</t>
+  </si>
+  <si>
+    <t>J1</t>
   </si>
 </sst>
 </file>
@@ -393,7 +414,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F160"/>
+  <dimension ref="A1:F162"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
@@ -2218,7 +2239,7 @@
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="B92">
         <v>1</v>
@@ -2226,39 +2247,21 @@
       <c r="C92" t="s">
         <v>4</v>
       </c>
-      <c r="D92">
-        <v>101</v>
-      </c>
-      <c r="E92">
-        <v>13</v>
-      </c>
-      <c r="F92" t="s">
-        <v>14</v>
-      </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="B93">
         <v>2</v>
       </c>
       <c r="C93" t="s">
         <v>4</v>
-      </c>
-      <c r="D93">
-        <v>67</v>
-      </c>
-      <c r="E93">
-        <v>1</v>
-      </c>
-      <c r="F93" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="B94">
         <v>3</v>
@@ -2266,39 +2269,21 @@
       <c r="C94" t="s">
         <v>4</v>
       </c>
-      <c r="D94">
-        <v>32</v>
-      </c>
-      <c r="E94">
-        <v>3</v>
-      </c>
-      <c r="F94" t="s">
-        <v>14</v>
-      </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="B95">
         <v>4</v>
       </c>
       <c r="C95" t="s">
         <v>4</v>
-      </c>
-      <c r="D95">
-        <v>99</v>
-      </c>
-      <c r="E95">
-        <v>11</v>
-      </c>
-      <c r="F95" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="B96">
         <v>5</v>
@@ -2306,19 +2291,10 @@
       <c r="C96" t="s">
         <v>4</v>
       </c>
-      <c r="D96">
-        <v>80</v>
-      </c>
-      <c r="E96">
-        <v>7</v>
-      </c>
-      <c r="F96" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="B97">
         <v>6</v>
@@ -2326,1274 +2302,720 @@
       <c r="C97" t="s">
         <v>4</v>
       </c>
-      <c r="D97">
-        <v>100</v>
-      </c>
-      <c r="E97">
+    </row>
+    <row r="98" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A98" t="s">
+        <v>15</v>
+      </c>
+      <c r="B98">
+        <v>7</v>
+      </c>
+      <c r="C98" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A99" t="s">
+        <v>15</v>
+      </c>
+      <c r="B99">
+        <v>8</v>
+      </c>
+      <c r="C99" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A100" t="s">
+        <v>15</v>
+      </c>
+      <c r="B100">
+        <v>9</v>
+      </c>
+      <c r="C100" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A101" t="s">
+        <v>15</v>
+      </c>
+      <c r="B101">
+        <v>10</v>
+      </c>
+      <c r="C101" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A102" t="s">
         <v>16</v>
       </c>
-      <c r="F97" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A98" t="s">
-        <v>7</v>
-      </c>
-      <c r="B98">
-        <v>7</v>
-      </c>
-      <c r="C98" t="s">
-        <v>4</v>
-      </c>
-      <c r="D98">
-        <v>96</v>
-      </c>
-      <c r="E98">
+      <c r="B102">
+        <v>1</v>
+      </c>
+      <c r="C102" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A103" t="s">
+        <v>16</v>
+      </c>
+      <c r="B103">
+        <v>2</v>
+      </c>
+      <c r="C103" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A104" t="s">
+        <v>16</v>
+      </c>
+      <c r="B104">
+        <v>3</v>
+      </c>
+      <c r="C104" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="105" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A105" t="s">
+        <v>16</v>
+      </c>
+      <c r="B105">
+        <v>4</v>
+      </c>
+      <c r="C105" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="106" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A106" t="s">
+        <v>16</v>
+      </c>
+      <c r="B106">
         <v>5</v>
       </c>
-      <c r="F98" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A99" t="s">
-        <v>7</v>
-      </c>
-      <c r="B99">
-        <v>8</v>
-      </c>
-      <c r="C99" t="s">
-        <v>4</v>
-      </c>
-      <c r="D99">
-        <v>95</v>
-      </c>
-      <c r="E99">
+      <c r="C106" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="107" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A107" t="s">
+        <v>16</v>
+      </c>
+      <c r="B107">
+        <v>6</v>
+      </c>
+      <c r="C107" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="108" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A108" t="s">
+        <v>16</v>
+      </c>
+      <c r="B108">
+        <v>7</v>
+      </c>
+      <c r="C108" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="109" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A109" t="s">
+        <v>16</v>
+      </c>
+      <c r="B109">
+        <v>8</v>
+      </c>
+      <c r="C109" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="110" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A110" t="s">
+        <v>16</v>
+      </c>
+      <c r="B110">
+        <v>9</v>
+      </c>
+      <c r="C110" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="111" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A111" t="s">
+        <v>16</v>
+      </c>
+      <c r="B111">
+        <v>10</v>
+      </c>
+      <c r="C111" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="112" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A112" t="s">
+        <v>16</v>
+      </c>
+      <c r="B112">
+        <v>11</v>
+      </c>
+      <c r="C112" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="113" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A113" t="s">
+        <v>17</v>
+      </c>
+      <c r="B113">
+        <v>1</v>
+      </c>
+      <c r="C113" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="114" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A114" t="s">
+        <v>17</v>
+      </c>
+      <c r="B114">
+        <v>2</v>
+      </c>
+      <c r="C114" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="115" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A115" t="s">
+        <v>17</v>
+      </c>
+      <c r="B115">
+        <v>3</v>
+      </c>
+      <c r="C115" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="116" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A116" t="s">
+        <v>17</v>
+      </c>
+      <c r="B116">
+        <v>4</v>
+      </c>
+      <c r="C116" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="117" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A117" t="s">
+        <v>17</v>
+      </c>
+      <c r="B117">
+        <v>5</v>
+      </c>
+      <c r="C117" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="118" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A118" t="s">
+        <v>17</v>
+      </c>
+      <c r="B118">
+        <v>6</v>
+      </c>
+      <c r="C118" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="119" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A119" t="s">
+        <v>17</v>
+      </c>
+      <c r="B119">
+        <v>7</v>
+      </c>
+      <c r="C119" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="120" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A120" t="s">
+        <v>17</v>
+      </c>
+      <c r="B120">
+        <v>8</v>
+      </c>
+      <c r="C120" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="121" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A121" t="s">
+        <v>17</v>
+      </c>
+      <c r="B121">
+        <v>9</v>
+      </c>
+      <c r="C121" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="122" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A122" t="s">
+        <v>17</v>
+      </c>
+      <c r="B122">
+        <v>10</v>
+      </c>
+      <c r="C122" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="123" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A123" t="s">
+        <v>18</v>
+      </c>
+      <c r="B123">
+        <v>1</v>
+      </c>
+      <c r="C123" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="124" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A124" t="s">
+        <v>18</v>
+      </c>
+      <c r="B124">
+        <v>2</v>
+      </c>
+      <c r="C124" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="125" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A125" t="s">
+        <v>18</v>
+      </c>
+      <c r="B125">
+        <v>3</v>
+      </c>
+      <c r="C125" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="126" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A126" t="s">
+        <v>18</v>
+      </c>
+      <c r="B126">
+        <v>4</v>
+      </c>
+      <c r="C126" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="127" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A127" t="s">
+        <v>18</v>
+      </c>
+      <c r="B127">
+        <v>5</v>
+      </c>
+      <c r="C127" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="128" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A128" t="s">
+        <v>18</v>
+      </c>
+      <c r="B128">
+        <v>6</v>
+      </c>
+      <c r="C128" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="129" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A129" t="s">
+        <v>18</v>
+      </c>
+      <c r="B129">
+        <v>7</v>
+      </c>
+      <c r="C129" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="130" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A130" t="s">
+        <v>18</v>
+      </c>
+      <c r="B130">
+        <v>8</v>
+      </c>
+      <c r="C130" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="131" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A131" t="s">
+        <v>18</v>
+      </c>
+      <c r="B131">
+        <v>9</v>
+      </c>
+      <c r="C131" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="132" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A132" t="s">
+        <v>18</v>
+      </c>
+      <c r="B132">
+        <v>10</v>
+      </c>
+      <c r="C132" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="133" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A133" t="s">
         <v>19</v>
       </c>
-      <c r="F99" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A100" t="s">
-        <v>7</v>
-      </c>
-      <c r="B100">
-        <v>11</v>
-      </c>
-      <c r="C100" t="s">
-        <v>4</v>
-      </c>
-      <c r="D100">
-        <v>95</v>
-      </c>
-      <c r="E100">
-        <v>13</v>
-      </c>
-      <c r="F100" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A101" t="s">
-        <v>6</v>
-      </c>
-      <c r="B101">
+      <c r="B133">
         <v>1</v>
       </c>
-      <c r="C101" t="s">
-        <v>4</v>
-      </c>
-      <c r="D101">
-        <v>137</v>
-      </c>
-      <c r="E101">
-        <v>73</v>
-      </c>
-      <c r="F101" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A102" t="s">
-        <v>6</v>
-      </c>
-      <c r="B102">
-        <v>2</v>
-      </c>
-      <c r="C102" t="s">
-        <v>4</v>
-      </c>
-      <c r="D102">
-        <v>112</v>
-      </c>
-      <c r="E102">
-        <v>69</v>
-      </c>
-      <c r="F102" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A103" t="s">
-        <v>6</v>
-      </c>
-      <c r="B103">
+      <c r="C133" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="134" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A134" t="s">
+        <v>19</v>
+      </c>
+      <c r="B134">
+        <v>2</v>
+      </c>
+      <c r="C134" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="135" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A135" t="s">
+        <v>19</v>
+      </c>
+      <c r="B135">
         <v>3</v>
       </c>
-      <c r="C103" t="s">
-        <v>4</v>
-      </c>
-      <c r="D103">
-        <v>91</v>
-      </c>
-      <c r="E103">
-        <v>48</v>
-      </c>
-      <c r="F103" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A104" t="s">
-        <v>6</v>
-      </c>
-      <c r="B104">
-        <v>4</v>
-      </c>
-      <c r="C104" t="s">
-        <v>4</v>
-      </c>
-      <c r="D104">
-        <v>55</v>
-      </c>
-      <c r="E104">
-        <v>44</v>
-      </c>
-      <c r="F104" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A105" t="s">
-        <v>6</v>
-      </c>
-      <c r="B105">
+      <c r="C135" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="136" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A136" t="s">
+        <v>19</v>
+      </c>
+      <c r="B136">
+        <v>4</v>
+      </c>
+      <c r="C136" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="137" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A137" t="s">
+        <v>19</v>
+      </c>
+      <c r="B137">
         <v>5</v>
       </c>
-      <c r="C105" t="s">
-        <v>4</v>
-      </c>
-      <c r="D105">
-        <v>88</v>
-      </c>
-      <c r="E105">
-        <v>63</v>
-      </c>
-      <c r="F105" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A106" t="s">
-        <v>6</v>
-      </c>
-      <c r="B106">
-        <v>6</v>
-      </c>
-      <c r="C106" t="s">
-        <v>4</v>
-      </c>
-      <c r="D106">
-        <v>125</v>
-      </c>
-      <c r="E106">
-        <v>67</v>
-      </c>
-      <c r="F106" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A107" t="s">
-        <v>6</v>
-      </c>
-      <c r="B107">
+      <c r="C137" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="138" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A138" t="s">
+        <v>19</v>
+      </c>
+      <c r="B138">
+        <v>6</v>
+      </c>
+      <c r="C138" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="139" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A139" t="s">
+        <v>19</v>
+      </c>
+      <c r="B139">
+        <v>7</v>
+      </c>
+      <c r="C139" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="140" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A140" t="s">
+        <v>19</v>
+      </c>
+      <c r="B140">
+        <v>8</v>
+      </c>
+      <c r="C140" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="141" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A141" t="s">
+        <v>19</v>
+      </c>
+      <c r="B141">
+        <v>9</v>
+      </c>
+      <c r="C141" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="142" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A142" t="s">
+        <v>19</v>
+      </c>
+      <c r="B142">
         <v>10</v>
       </c>
-      <c r="C107" t="s">
-        <v>4</v>
-      </c>
-      <c r="D107">
-        <v>83</v>
-      </c>
-      <c r="E107">
-        <v>31</v>
-      </c>
-      <c r="F107" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A108" t="s">
-        <v>6</v>
-      </c>
-      <c r="B108">
-        <v>11</v>
-      </c>
-      <c r="C108" t="s">
-        <v>4</v>
-      </c>
-      <c r="D108">
-        <v>83</v>
-      </c>
-      <c r="E108">
-        <v>53</v>
-      </c>
-      <c r="F108" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A109" t="s">
-        <v>8</v>
-      </c>
-      <c r="B109">
+      <c r="C142" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="143" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A143" t="s">
+        <v>20</v>
+      </c>
+      <c r="B143">
         <v>1</v>
       </c>
-      <c r="C109" t="s">
-        <v>4</v>
-      </c>
-      <c r="D109">
-        <v>81</v>
-      </c>
-      <c r="E109">
+      <c r="C143" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="144" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A144" t="s">
+        <v>20</v>
+      </c>
+      <c r="B144">
+        <v>2</v>
+      </c>
+      <c r="C144" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="145" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A145" t="s">
+        <v>20</v>
+      </c>
+      <c r="B145">
+        <v>3</v>
+      </c>
+      <c r="C145" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="146" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A146" t="s">
+        <v>20</v>
+      </c>
+      <c r="B146">
+        <v>4</v>
+      </c>
+      <c r="C146" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="147" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A147" t="s">
+        <v>20</v>
+      </c>
+      <c r="B147">
+        <v>5</v>
+      </c>
+      <c r="C147" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="148" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A148" t="s">
+        <v>20</v>
+      </c>
+      <c r="B148">
+        <v>6</v>
+      </c>
+      <c r="C148" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="149" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A149" t="s">
+        <v>20</v>
+      </c>
+      <c r="B149">
+        <v>7</v>
+      </c>
+      <c r="C149" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="150" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A150" t="s">
+        <v>20</v>
+      </c>
+      <c r="B150">
+        <v>8</v>
+      </c>
+      <c r="C150" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="151" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A151" t="s">
+        <v>20</v>
+      </c>
+      <c r="B151">
         <v>9</v>
       </c>
-      <c r="F109" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A110" t="s">
-        <v>8</v>
-      </c>
-      <c r="B110">
-        <v>2</v>
-      </c>
-      <c r="C110" t="s">
-        <v>4</v>
-      </c>
-      <c r="D110">
-        <v>81</v>
-      </c>
-      <c r="E110">
-        <v>4</v>
-      </c>
-      <c r="F110" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A111" t="s">
-        <v>8</v>
-      </c>
-      <c r="B111">
+      <c r="C151" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="152" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A152" t="s">
+        <v>20</v>
+      </c>
+      <c r="B152">
+        <v>10</v>
+      </c>
+      <c r="C152" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="153" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A153" t="s">
+        <v>21</v>
+      </c>
+      <c r="B153">
+        <v>1</v>
+      </c>
+      <c r="C153" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="154" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A154" t="s">
+        <v>21</v>
+      </c>
+      <c r="B154">
+        <v>2</v>
+      </c>
+      <c r="C154" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="155" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A155" t="s">
+        <v>21</v>
+      </c>
+      <c r="B155">
         <v>3</v>
       </c>
-      <c r="C111" t="s">
-        <v>4</v>
-      </c>
-      <c r="D111">
-        <v>112</v>
-      </c>
-      <c r="E111">
-        <v>11</v>
-      </c>
-      <c r="F111" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A112" t="s">
-        <v>8</v>
-      </c>
-      <c r="B112">
+      <c r="C155" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="156" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A156" t="s">
+        <v>21</v>
+      </c>
+      <c r="B156">
+        <v>4</v>
+      </c>
+      <c r="C156" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="157" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A157" t="s">
+        <v>21</v>
+      </c>
+      <c r="B157">
         <v>5</v>
       </c>
-      <c r="C112" t="s">
-        <v>4</v>
-      </c>
-      <c r="D112">
-        <v>80</v>
-      </c>
-      <c r="E112">
+      <c r="C157" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="158" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A158" t="s">
+        <v>21</v>
+      </c>
+      <c r="B158">
+        <v>6</v>
+      </c>
+      <c r="C158" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="159" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A159" t="s">
+        <v>21</v>
+      </c>
+      <c r="B159">
+        <v>7</v>
+      </c>
+      <c r="C159" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="160" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A160" t="s">
+        <v>21</v>
+      </c>
+      <c r="B160">
+        <v>8</v>
+      </c>
+      <c r="C160" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="161" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A161" t="s">
+        <v>21</v>
+      </c>
+      <c r="B161">
+        <v>9</v>
+      </c>
+      <c r="C161" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="162" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A162" t="s">
+        <v>21</v>
+      </c>
+      <c r="B162">
         <v>10</v>
       </c>
-      <c r="F112" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A113" t="s">
-        <v>8</v>
-      </c>
-      <c r="B113">
-        <v>6</v>
-      </c>
-      <c r="C113" t="s">
-        <v>4</v>
-      </c>
-      <c r="D113">
-        <v>70</v>
-      </c>
-      <c r="E113">
-        <v>5</v>
-      </c>
-      <c r="F113" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A114" t="s">
-        <v>8</v>
-      </c>
-      <c r="B114">
-        <v>7</v>
-      </c>
-      <c r="C114" t="s">
-        <v>4</v>
-      </c>
-      <c r="D114">
-        <v>34</v>
-      </c>
-      <c r="E114">
-        <v>4</v>
-      </c>
-      <c r="F114" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A115" t="s">
-        <v>8</v>
-      </c>
-      <c r="B115">
-        <v>8</v>
-      </c>
-      <c r="C115" t="s">
-        <v>4</v>
-      </c>
-      <c r="D115">
-        <v>91</v>
-      </c>
-      <c r="E115">
-        <v>2</v>
-      </c>
-      <c r="F115" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A116" t="s">
-        <v>8</v>
-      </c>
-      <c r="B116">
-        <v>9</v>
-      </c>
-      <c r="C116" t="s">
-        <v>4</v>
-      </c>
-      <c r="D116">
-        <v>89</v>
-      </c>
-      <c r="E116">
-        <v>3</v>
-      </c>
-      <c r="F116" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A117" t="s">
-        <v>8</v>
-      </c>
-      <c r="B117">
-        <v>10</v>
-      </c>
-      <c r="C117" t="s">
-        <v>4</v>
-      </c>
-      <c r="D117">
-        <v>71</v>
-      </c>
-      <c r="E117">
-        <v>9</v>
-      </c>
-      <c r="F117" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A118" t="s">
-        <v>8</v>
-      </c>
-      <c r="B118">
-        <v>11</v>
-      </c>
-      <c r="C118" t="s">
-        <v>4</v>
-      </c>
-      <c r="D118">
-        <v>85</v>
-      </c>
-      <c r="E118">
-        <v>7</v>
-      </c>
-      <c r="F118" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A119" t="s">
-        <v>2</v>
-      </c>
-      <c r="B119">
-        <v>1</v>
-      </c>
-      <c r="C119" t="s">
-        <v>11</v>
-      </c>
-      <c r="D119">
-        <v>175</v>
-      </c>
-      <c r="E119">
-        <v>6</v>
-      </c>
-      <c r="F119" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A120" t="s">
-        <v>2</v>
-      </c>
-      <c r="B120">
-        <v>2</v>
-      </c>
-      <c r="C120" t="s">
-        <v>11</v>
-      </c>
-      <c r="D120">
-        <v>96</v>
-      </c>
-      <c r="E120">
-        <v>1</v>
-      </c>
-      <c r="F120" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A121" t="s">
-        <v>2</v>
-      </c>
-      <c r="B121">
-        <v>3</v>
-      </c>
-      <c r="C121" t="s">
-        <v>11</v>
-      </c>
-      <c r="D121">
-        <v>99</v>
-      </c>
-      <c r="E121">
-        <v>1</v>
-      </c>
-      <c r="F121" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A122" t="s">
-        <v>2</v>
-      </c>
-      <c r="B122">
-        <v>4</v>
-      </c>
-      <c r="C122" t="s">
-        <v>11</v>
-      </c>
-      <c r="D122">
-        <v>105</v>
-      </c>
-      <c r="E122">
-        <v>2</v>
-      </c>
-      <c r="F122" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A123" t="s">
-        <v>2</v>
-      </c>
-      <c r="B123">
-        <v>5</v>
-      </c>
-      <c r="C123" t="s">
-        <v>11</v>
-      </c>
-      <c r="D123">
-        <v>129</v>
-      </c>
-      <c r="E123">
-        <v>8</v>
-      </c>
-      <c r="F123" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A124" t="s">
-        <v>2</v>
-      </c>
-      <c r="B124">
-        <v>6</v>
-      </c>
-      <c r="C124" t="s">
-        <v>11</v>
-      </c>
-      <c r="D124">
-        <v>148</v>
-      </c>
-      <c r="E124">
-        <v>5</v>
-      </c>
-      <c r="F124" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A125" t="s">
-        <v>2</v>
-      </c>
-      <c r="B125">
-        <v>7</v>
-      </c>
-      <c r="C125" t="s">
-        <v>11</v>
-      </c>
-      <c r="D125">
-        <v>138</v>
-      </c>
-      <c r="E125">
-        <v>5</v>
-      </c>
-      <c r="F125" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A126" t="s">
-        <v>2</v>
-      </c>
-      <c r="B126">
-        <v>8</v>
-      </c>
-      <c r="C126" t="s">
-        <v>11</v>
-      </c>
-      <c r="D126">
-        <v>138</v>
-      </c>
-      <c r="E126">
-        <v>14</v>
-      </c>
-      <c r="F126" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A127" t="s">
-        <v>2</v>
-      </c>
-      <c r="B127">
-        <v>9</v>
-      </c>
-      <c r="C127" t="s">
-        <v>11</v>
-      </c>
-      <c r="D127">
-        <v>158</v>
-      </c>
-      <c r="E127">
-        <v>6</v>
-      </c>
-      <c r="F127" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A128" t="s">
-        <v>2</v>
-      </c>
-      <c r="B128">
-        <v>10</v>
-      </c>
-      <c r="C128" t="s">
-        <v>11</v>
-      </c>
-      <c r="D128">
-        <v>166</v>
-      </c>
-      <c r="E128">
-        <v>6</v>
-      </c>
-      <c r="F128" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A129" t="s">
-        <v>2</v>
-      </c>
-      <c r="B129">
-        <v>11</v>
-      </c>
-      <c r="C129" t="s">
-        <v>11</v>
-      </c>
-      <c r="D129">
-        <v>95</v>
-      </c>
-      <c r="E129">
-        <v>4</v>
-      </c>
-      <c r="F129" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A130" t="s">
-        <v>6</v>
-      </c>
-      <c r="B130">
-        <v>1</v>
-      </c>
-      <c r="C130" t="s">
-        <v>11</v>
-      </c>
-      <c r="D130">
-        <v>77</v>
-      </c>
-      <c r="E130">
-        <v>1</v>
-      </c>
-      <c r="F130" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A131" t="s">
-        <v>6</v>
-      </c>
-      <c r="B131">
-        <v>2</v>
-      </c>
-      <c r="C131" t="s">
-        <v>11</v>
-      </c>
-      <c r="D131">
-        <v>101</v>
-      </c>
-      <c r="E131">
-        <v>5</v>
-      </c>
-      <c r="F131" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A132" t="s">
-        <v>6</v>
-      </c>
-      <c r="B132">
-        <v>3</v>
-      </c>
-      <c r="C132" t="s">
-        <v>11</v>
-      </c>
-      <c r="D132">
-        <v>153</v>
-      </c>
-      <c r="E132">
-        <v>0</v>
-      </c>
-      <c r="F132" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A133" t="s">
-        <v>6</v>
-      </c>
-      <c r="B133">
-        <v>4</v>
-      </c>
-      <c r="C133" t="s">
-        <v>11</v>
-      </c>
-      <c r="D133">
-        <v>103</v>
-      </c>
-      <c r="E133">
-        <v>3</v>
-      </c>
-      <c r="F133" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A134" t="s">
-        <v>6</v>
-      </c>
-      <c r="B134">
-        <v>5</v>
-      </c>
-      <c r="C134" t="s">
-        <v>11</v>
-      </c>
-      <c r="D134">
-        <v>97</v>
-      </c>
-      <c r="E134">
-        <v>4</v>
-      </c>
-      <c r="F134" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A135" t="s">
-        <v>6</v>
-      </c>
-      <c r="B135">
-        <v>6</v>
-      </c>
-      <c r="C135" t="s">
-        <v>11</v>
-      </c>
-      <c r="D135">
-        <v>111</v>
-      </c>
-      <c r="E135">
-        <v>3</v>
-      </c>
-      <c r="F135" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A136" t="s">
-        <v>6</v>
-      </c>
-      <c r="B136">
-        <v>7</v>
-      </c>
-      <c r="C136" t="s">
-        <v>11</v>
-      </c>
-      <c r="D136">
-        <v>179</v>
-      </c>
-      <c r="E136">
-        <v>10</v>
-      </c>
-      <c r="F136" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A137" t="s">
-        <v>6</v>
-      </c>
-      <c r="B137">
-        <v>8</v>
-      </c>
-      <c r="C137" t="s">
-        <v>11</v>
-      </c>
-      <c r="D137">
-        <v>84</v>
-      </c>
-      <c r="E137">
-        <v>9</v>
-      </c>
-      <c r="F137" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A138" t="s">
-        <v>6</v>
-      </c>
-      <c r="B138">
-        <v>9</v>
-      </c>
-      <c r="C138" t="s">
-        <v>11</v>
-      </c>
-      <c r="D138">
-        <v>198</v>
-      </c>
-      <c r="E138">
-        <v>12</v>
-      </c>
-      <c r="F138" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A139" t="s">
-        <v>6</v>
-      </c>
-      <c r="B139">
-        <v>10</v>
-      </c>
-      <c r="C139" t="s">
-        <v>11</v>
-      </c>
-      <c r="D139">
-        <v>113</v>
-      </c>
-      <c r="E139">
-        <v>5</v>
-      </c>
-      <c r="F139" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A140" t="s">
-        <v>6</v>
-      </c>
-      <c r="B140">
-        <v>11</v>
-      </c>
-      <c r="C140" t="s">
-        <v>11</v>
-      </c>
-      <c r="D140">
-        <v>127</v>
-      </c>
-      <c r="E140">
-        <v>10</v>
-      </c>
-      <c r="F140" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A141" t="s">
-        <v>7</v>
-      </c>
-      <c r="B141">
-        <v>1</v>
-      </c>
-      <c r="C141" t="s">
-        <v>11</v>
-      </c>
-      <c r="D141">
-        <v>128</v>
-      </c>
-      <c r="E141">
-        <v>0</v>
-      </c>
-      <c r="F141" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A142" t="s">
-        <v>7</v>
-      </c>
-      <c r="B142">
-        <v>2</v>
-      </c>
-      <c r="C142" t="s">
-        <v>11</v>
-      </c>
-      <c r="D142">
-        <v>106</v>
-      </c>
-      <c r="E142">
-        <v>0</v>
-      </c>
-      <c r="F142" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A143" t="s">
-        <v>7</v>
-      </c>
-      <c r="B143">
-        <v>3</v>
-      </c>
-      <c r="C143" t="s">
-        <v>11</v>
-      </c>
-      <c r="D143">
-        <v>92</v>
-      </c>
-      <c r="E143">
-        <v>1</v>
-      </c>
-      <c r="F143" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A144" t="s">
-        <v>7</v>
-      </c>
-      <c r="B144">
-        <v>4</v>
-      </c>
-      <c r="C144" t="s">
-        <v>11</v>
-      </c>
-      <c r="D144">
-        <v>78</v>
-      </c>
-      <c r="E144">
-        <v>0</v>
-      </c>
-      <c r="F144" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A145" t="s">
-        <v>7</v>
-      </c>
-      <c r="B145">
-        <v>5</v>
-      </c>
-      <c r="C145" t="s">
-        <v>11</v>
-      </c>
-      <c r="D145">
-        <v>84</v>
-      </c>
-      <c r="E145">
-        <v>0</v>
-      </c>
-      <c r="F145" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A146" t="s">
-        <v>7</v>
-      </c>
-      <c r="B146">
-        <v>6</v>
-      </c>
-      <c r="C146" t="s">
-        <v>11</v>
-      </c>
-      <c r="D146">
-        <v>129</v>
-      </c>
-      <c r="E146">
-        <v>0</v>
-      </c>
-      <c r="F146" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="147" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A147" t="s">
-        <v>7</v>
-      </c>
-      <c r="B147">
-        <v>7</v>
-      </c>
-      <c r="C147" t="s">
-        <v>11</v>
-      </c>
-      <c r="D147">
-        <v>69</v>
-      </c>
-      <c r="E147">
-        <v>0</v>
-      </c>
-      <c r="F147" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="148" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A148" t="s">
-        <v>7</v>
-      </c>
-      <c r="B148">
-        <v>8</v>
-      </c>
-      <c r="C148" t="s">
-        <v>11</v>
-      </c>
-      <c r="D148">
-        <v>119</v>
-      </c>
-      <c r="E148">
-        <v>0</v>
-      </c>
-      <c r="F148" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="149" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A149" t="s">
-        <v>7</v>
-      </c>
-      <c r="B149">
-        <v>9</v>
-      </c>
-      <c r="C149" t="s">
-        <v>11</v>
-      </c>
-      <c r="D149">
-        <v>97</v>
-      </c>
-      <c r="E149">
-        <v>0</v>
-      </c>
-      <c r="F149" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="150" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A150" t="s">
-        <v>7</v>
-      </c>
-      <c r="B150">
-        <v>10</v>
-      </c>
-      <c r="C150" t="s">
-        <v>11</v>
-      </c>
-      <c r="D150">
-        <v>147</v>
-      </c>
-      <c r="E150">
-        <v>0</v>
-      </c>
-      <c r="F150" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="151" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A151" t="s">
-        <v>8</v>
-      </c>
-      <c r="B151">
-        <v>1</v>
-      </c>
-      <c r="C151" t="s">
-        <v>11</v>
-      </c>
-      <c r="D151">
-        <v>100</v>
-      </c>
-      <c r="E151">
-        <v>0</v>
-      </c>
-      <c r="F151" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="152" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A152" t="s">
-        <v>8</v>
-      </c>
-      <c r="B152">
-        <v>2</v>
-      </c>
-      <c r="C152" t="s">
-        <v>11</v>
-      </c>
-      <c r="D152">
-        <v>124</v>
-      </c>
-      <c r="E152">
-        <v>0</v>
-      </c>
-      <c r="F152" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="153" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A153" t="s">
-        <v>8</v>
-      </c>
-      <c r="B153">
-        <v>3</v>
-      </c>
-      <c r="C153" t="s">
-        <v>11</v>
-      </c>
-      <c r="D153">
-        <v>80</v>
-      </c>
-      <c r="E153">
-        <v>0</v>
-      </c>
-      <c r="F153" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="154" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A154" t="s">
-        <v>8</v>
-      </c>
-      <c r="B154">
-        <v>4</v>
-      </c>
-      <c r="C154" t="s">
-        <v>11</v>
-      </c>
-      <c r="D154">
-        <v>83</v>
-      </c>
-      <c r="E154">
-        <v>0</v>
-      </c>
-      <c r="F154" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="155" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A155" t="s">
-        <v>8</v>
-      </c>
-      <c r="B155">
-        <v>5</v>
-      </c>
-      <c r="C155" t="s">
-        <v>11</v>
-      </c>
-      <c r="D155">
-        <v>110</v>
-      </c>
-      <c r="E155">
-        <v>2</v>
-      </c>
-      <c r="F155" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="156" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A156" t="s">
-        <v>8</v>
-      </c>
-      <c r="B156">
-        <v>6</v>
-      </c>
-      <c r="C156" t="s">
-        <v>11</v>
-      </c>
-      <c r="D156">
-        <v>184</v>
-      </c>
-      <c r="E156">
-        <v>0</v>
-      </c>
-      <c r="F156" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="157" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A157" t="s">
-        <v>8</v>
-      </c>
-      <c r="B157">
-        <v>7</v>
-      </c>
-      <c r="C157" t="s">
-        <v>11</v>
-      </c>
-      <c r="D157">
-        <v>132</v>
-      </c>
-      <c r="E157">
-        <v>0</v>
-      </c>
-      <c r="F157" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="158" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A158" t="s">
-        <v>8</v>
-      </c>
-      <c r="B158">
-        <v>8</v>
-      </c>
-      <c r="C158" t="s">
-        <v>11</v>
-      </c>
-      <c r="D158">
-        <v>114</v>
-      </c>
-      <c r="E158">
-        <v>0</v>
-      </c>
-      <c r="F158" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="159" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A159" t="s">
-        <v>8</v>
-      </c>
-      <c r="B159">
-        <v>9</v>
-      </c>
-      <c r="C159" t="s">
-        <v>11</v>
-      </c>
-      <c r="D159">
-        <v>122</v>
-      </c>
-      <c r="E159">
-        <v>0</v>
-      </c>
-      <c r="F159" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="160" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A160" t="s">
-        <v>8</v>
-      </c>
-      <c r="B160">
-        <v>10</v>
-      </c>
-      <c r="C160" t="s">
-        <v>11</v>
-      </c>
-      <c r="D160">
-        <v>69</v>
-      </c>
-      <c r="E160">
-        <v>0</v>
-      </c>
-      <c r="F160" t="s">
-        <v>14</v>
+      <c r="C162" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
cell counts for G-J
</commit_message>
<xml_diff>
--- a/data/raw/Cell_Counts/Dazl_100nMRA/241009_Dazl_100nMRA.xlsx
+++ b/data/raw/Cell_Counts/Dazl_100nMRA/241009_Dazl_100nMRA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://umhealth-my.sharepoint.com/personal/kbonefas_med_umich_edu/Documents/Documents/KDM5C_Germ_Mechanism/data/raw/Cell_Counts/Dazl_100nMRA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="542" documentId="11_F25DC773A252ABDACC1048D6E9986E465BDE58ED" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4D9271E9-4378-4154-BE31-D00EFEE944CE}"/>
+  <xr:revisionPtr revIDLastSave="711" documentId="11_F25DC773A252ABDACC1048D6E9986E465BDE58ED" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BBE90E81-E5D9-4226-AA88-AA7625A8DF8F}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10530" yWindow="680" windowWidth="9740" windowHeight="8890" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="418" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="420" uniqueCount="22">
   <si>
     <t>Image</t>
   </si>
@@ -149,6 +149,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -414,7 +418,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F162"/>
+  <dimension ref="A1:F163"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
@@ -2247,6 +2251,12 @@
       <c r="C92" t="s">
         <v>4</v>
       </c>
+      <c r="D92">
+        <v>45</v>
+      </c>
+      <c r="E92">
+        <v>34</v>
+      </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
@@ -2258,6 +2268,12 @@
       <c r="C93" t="s">
         <v>4</v>
       </c>
+      <c r="D93">
+        <v>76</v>
+      </c>
+      <c r="E93">
+        <v>41</v>
+      </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
@@ -2269,6 +2285,12 @@
       <c r="C94" t="s">
         <v>4</v>
       </c>
+      <c r="D94">
+        <v>68</v>
+      </c>
+      <c r="E94">
+        <v>39</v>
+      </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
@@ -2280,6 +2302,12 @@
       <c r="C95" t="s">
         <v>4</v>
       </c>
+      <c r="D95">
+        <v>67</v>
+      </c>
+      <c r="E95">
+        <v>53</v>
+      </c>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
@@ -2291,8 +2319,14 @@
       <c r="C96" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D96">
+        <v>59</v>
+      </c>
+      <c r="E96">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>15</v>
       </c>
@@ -2302,8 +2336,14 @@
       <c r="C97" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D97">
+        <v>70</v>
+      </c>
+      <c r="E97">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>15</v>
       </c>
@@ -2313,8 +2353,14 @@
       <c r="C98" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D98">
+        <v>66</v>
+      </c>
+      <c r="E98">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>15</v>
       </c>
@@ -2324,8 +2370,14 @@
       <c r="C99" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D99">
+        <v>83</v>
+      </c>
+      <c r="E99">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>15</v>
       </c>
@@ -2335,8 +2387,14 @@
       <c r="C100" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D100">
+        <v>96</v>
+      </c>
+      <c r="E100">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>15</v>
       </c>
@@ -2346,8 +2404,14 @@
       <c r="C101" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D101">
+        <v>56</v>
+      </c>
+      <c r="E101">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>16</v>
       </c>
@@ -2357,8 +2421,14 @@
       <c r="C102" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D102">
+        <v>87</v>
+      </c>
+      <c r="E102">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>16</v>
       </c>
@@ -2368,8 +2438,14 @@
       <c r="C103" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D103">
+        <v>100</v>
+      </c>
+      <c r="E103">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
         <v>16</v>
       </c>
@@ -2379,8 +2455,14 @@
       <c r="C104" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D104">
+        <v>91</v>
+      </c>
+      <c r="E104">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
         <v>16</v>
       </c>
@@ -2390,8 +2472,14 @@
       <c r="C105" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D105">
+        <v>86</v>
+      </c>
+      <c r="E105">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
         <v>16</v>
       </c>
@@ -2401,8 +2489,14 @@
       <c r="C106" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D106">
+        <v>68</v>
+      </c>
+      <c r="E106">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
         <v>16</v>
       </c>
@@ -2412,8 +2506,14 @@
       <c r="C107" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D107">
+        <v>149</v>
+      </c>
+      <c r="E107">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
         <v>16</v>
       </c>
@@ -2423,8 +2523,14 @@
       <c r="C108" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D108">
+        <v>76</v>
+      </c>
+      <c r="E108">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
         <v>16</v>
       </c>
@@ -2434,8 +2540,14 @@
       <c r="C109" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D109">
+        <v>86</v>
+      </c>
+      <c r="E109">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="110" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
         <v>16</v>
       </c>
@@ -2445,8 +2557,14 @@
       <c r="C110" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D110">
+        <v>82</v>
+      </c>
+      <c r="E110">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="111" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
         <v>16</v>
       </c>
@@ -2456,8 +2574,14 @@
       <c r="C111" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D111">
+        <v>63</v>
+      </c>
+      <c r="E111">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="112" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
         <v>16</v>
       </c>
@@ -2467,8 +2591,14 @@
       <c r="C112" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D112">
+        <v>51</v>
+      </c>
+      <c r="E112">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
         <v>17</v>
       </c>
@@ -2478,8 +2608,14 @@
       <c r="C113" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D113">
+        <v>50</v>
+      </c>
+      <c r="E113">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
         <v>17</v>
       </c>
@@ -2489,8 +2625,14 @@
       <c r="C114" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D114">
+        <v>40</v>
+      </c>
+      <c r="E114">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
         <v>17</v>
       </c>
@@ -2500,8 +2642,14 @@
       <c r="C115" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="116" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D115">
+        <v>53</v>
+      </c>
+      <c r="E115">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
         <v>17</v>
       </c>
@@ -2511,8 +2659,14 @@
       <c r="C116" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="117" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D116">
+        <v>37</v>
+      </c>
+      <c r="E116">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
         <v>17</v>
       </c>
@@ -2522,8 +2676,14 @@
       <c r="C117" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="118" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D117">
+        <v>44</v>
+      </c>
+      <c r="E117">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
         <v>17</v>
       </c>
@@ -2533,8 +2693,14 @@
       <c r="C118" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="119" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D118">
+        <v>53</v>
+      </c>
+      <c r="E118">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
         <v>17</v>
       </c>
@@ -2544,8 +2710,14 @@
       <c r="C119" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="120" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D119">
+        <v>43</v>
+      </c>
+      <c r="E119">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
         <v>17</v>
       </c>
@@ -2555,8 +2727,14 @@
       <c r="C120" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="121" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D120">
+        <v>59</v>
+      </c>
+      <c r="E120">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
         <v>17</v>
       </c>
@@ -2566,8 +2744,14 @@
       <c r="C121" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="122" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D121">
+        <v>28</v>
+      </c>
+      <c r="E121">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
         <v>17</v>
       </c>
@@ -2577,8 +2761,14 @@
       <c r="C122" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="123" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D122">
+        <v>53</v>
+      </c>
+      <c r="E122">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
         <v>18</v>
       </c>
@@ -2588,8 +2778,14 @@
       <c r="C123" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="124" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D123">
+        <v>67</v>
+      </c>
+      <c r="E123">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
         <v>18</v>
       </c>
@@ -2599,8 +2795,14 @@
       <c r="C124" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="125" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D124">
+        <v>91</v>
+      </c>
+      <c r="E124">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
         <v>18</v>
       </c>
@@ -2610,8 +2812,14 @@
       <c r="C125" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="126" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D125">
+        <v>154</v>
+      </c>
+      <c r="E125">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="126" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
         <v>18</v>
       </c>
@@ -2621,8 +2829,14 @@
       <c r="C126" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="127" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D126">
+        <v>34</v>
+      </c>
+      <c r="E126">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="127" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
         <v>18</v>
       </c>
@@ -2632,8 +2846,14 @@
       <c r="C127" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="128" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D127">
+        <v>132</v>
+      </c>
+      <c r="E127">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="128" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
         <v>18</v>
       </c>
@@ -2643,8 +2863,14 @@
       <c r="C128" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="129" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D128">
+        <v>129</v>
+      </c>
+      <c r="E128">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
         <v>18</v>
       </c>
@@ -2654,8 +2880,14 @@
       <c r="C129" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="130" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D129">
+        <v>84</v>
+      </c>
+      <c r="E129">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="130" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A130" t="s">
         <v>18</v>
       </c>
@@ -2665,8 +2897,14 @@
       <c r="C130" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="131" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D130">
+        <v>144</v>
+      </c>
+      <c r="E130">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="131" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
         <v>18</v>
       </c>
@@ -2676,8 +2914,14 @@
       <c r="C131" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="132" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D131">
+        <v>89</v>
+      </c>
+      <c r="E131">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="132" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
         <v>18</v>
       </c>
@@ -2687,8 +2931,14 @@
       <c r="C132" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="133" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D132">
+        <v>71</v>
+      </c>
+      <c r="E132">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="133" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
         <v>19</v>
       </c>
@@ -2698,8 +2948,14 @@
       <c r="C133" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="134" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D133">
+        <v>134</v>
+      </c>
+      <c r="E133">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="134" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
         <v>19</v>
       </c>
@@ -2709,8 +2965,14 @@
       <c r="C134" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="135" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D134">
+        <v>191</v>
+      </c>
+      <c r="E134">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="135" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
         <v>19</v>
       </c>
@@ -2720,8 +2982,14 @@
       <c r="C135" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="136" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D135">
+        <v>131</v>
+      </c>
+      <c r="E135">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="136" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
         <v>19</v>
       </c>
@@ -2731,8 +2999,14 @@
       <c r="C136" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="137" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D136">
+        <v>90</v>
+      </c>
+      <c r="E136">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="137" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
         <v>19</v>
       </c>
@@ -2742,8 +3016,14 @@
       <c r="C137" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="138" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D137">
+        <v>116</v>
+      </c>
+      <c r="E137">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="138" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
         <v>19</v>
       </c>
@@ -2753,8 +3033,14 @@
       <c r="C138" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="139" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D138">
+        <v>196</v>
+      </c>
+      <c r="E138">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="139" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
         <v>19</v>
       </c>
@@ -2764,8 +3050,14 @@
       <c r="C139" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="140" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D139">
+        <v>131</v>
+      </c>
+      <c r="E139">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="140" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
         <v>19</v>
       </c>
@@ -2775,8 +3067,14 @@
       <c r="C140" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="141" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D140">
+        <v>142</v>
+      </c>
+      <c r="E140">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="141" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A141" t="s">
         <v>19</v>
       </c>
@@ -2786,8 +3084,14 @@
       <c r="C141" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="142" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D141">
+        <v>157</v>
+      </c>
+      <c r="E141">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="142" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A142" t="s">
         <v>19</v>
       </c>
@@ -2797,217 +3101,337 @@
       <c r="C142" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="143" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D142">
+        <v>170</v>
+      </c>
+      <c r="E142">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="143" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A143" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B143">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C143" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="144" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D143">
+        <v>111</v>
+      </c>
+      <c r="E143">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="144" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A144" t="s">
         <v>20</v>
       </c>
       <c r="B144">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C144" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="145" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D144">
+        <v>189</v>
+      </c>
+      <c r="E144">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="145" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A145" t="s">
         <v>20</v>
       </c>
       <c r="B145">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C145" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="146" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D145">
+        <v>110</v>
+      </c>
+      <c r="E145">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="146" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A146" t="s">
         <v>20</v>
       </c>
       <c r="B146">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C146" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="147" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D146">
+        <v>115</v>
+      </c>
+      <c r="E146">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="147" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A147" t="s">
         <v>20</v>
       </c>
       <c r="B147">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C147" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="148" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D147">
+        <v>142</v>
+      </c>
+      <c r="E147">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="148" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A148" t="s">
         <v>20</v>
       </c>
       <c r="B148">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C148" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="149" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D148">
+        <v>102</v>
+      </c>
+      <c r="E148">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="149" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A149" t="s">
         <v>20</v>
       </c>
       <c r="B149">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C149" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="150" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D149">
+        <v>155</v>
+      </c>
+      <c r="E149">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="150" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A150" t="s">
         <v>20</v>
       </c>
       <c r="B150">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C150" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="151" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D150">
+        <v>114</v>
+      </c>
+      <c r="E150">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="151" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A151" t="s">
         <v>20</v>
       </c>
       <c r="B151">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C151" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="152" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D151">
+        <v>208</v>
+      </c>
+      <c r="E151">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="152" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A152" t="s">
         <v>20</v>
       </c>
       <c r="B152">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C152" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="153" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D152">
+        <v>203</v>
+      </c>
+      <c r="E152">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="153" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A153" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B153">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C153" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="154" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D153">
+        <v>205</v>
+      </c>
+      <c r="E153">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="154" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A154" t="s">
         <v>21</v>
       </c>
       <c r="B154">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C154" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="155" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D154">
+        <v>77</v>
+      </c>
+      <c r="E154">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="155" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A155" t="s">
         <v>21</v>
       </c>
       <c r="B155">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C155" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="156" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D155">
+        <v>97</v>
+      </c>
+      <c r="E155">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="156" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A156" t="s">
         <v>21</v>
       </c>
       <c r="B156">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C156" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="157" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D156">
+        <v>149</v>
+      </c>
+      <c r="E156">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="157" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A157" t="s">
         <v>21</v>
       </c>
       <c r="B157">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C157" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="158" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D157">
+        <v>71</v>
+      </c>
+      <c r="E157">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="158" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A158" t="s">
         <v>21</v>
       </c>
       <c r="B158">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C158" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="159" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D158">
+        <v>108</v>
+      </c>
+      <c r="E158">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="159" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A159" t="s">
         <v>21</v>
       </c>
       <c r="B159">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C159" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="160" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D159">
+        <v>50</v>
+      </c>
+      <c r="E159">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="160" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A160" t="s">
         <v>21</v>
       </c>
       <c r="B160">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C160" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="161" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D160">
+        <v>110</v>
+      </c>
+      <c r="E160">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="161" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A161" t="s">
         <v>21</v>
       </c>
       <c r="B161">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C161" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="162" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D161">
+        <v>95</v>
+      </c>
+      <c r="E161">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="162" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A162" t="s">
         <v>21</v>
       </c>
@@ -3016,6 +3440,29 @@
       </c>
       <c r="C162" t="s">
         <v>11</v>
+      </c>
+      <c r="D162">
+        <v>155</v>
+      </c>
+      <c r="E162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="163" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A163" t="s">
+        <v>21</v>
+      </c>
+      <c r="B163">
+        <v>11</v>
+      </c>
+      <c r="C163" t="s">
+        <v>11</v>
+      </c>
+      <c r="D163">
+        <v>106</v>
+      </c>
+      <c r="E163">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>